<commit_message>
updated functionality for archival objects
</commit_message>
<xml_diff>
--- a/docs/sample_data.xlsx
+++ b/docs/sample_data.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10409"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/steffen/git/goobi-workflow/plugin-import-eth-no-catalogue/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/steffen/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4CE04156-37B3-5240-A247-5B2E2A2C3D0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4D92E553-9DE4-D046-B3AB-825870DF869B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4360" yWindow="3760" windowWidth="27040" windowHeight="15740" xr2:uid="{799CE81A-27C5-664D-9EEE-5BE1EC197E54}"/>
+    <workbookView xWindow="-2000" yWindow="-21580" windowWidth="27840" windowHeight="16740" xr2:uid="{B1ADD6CB-816E-0D4F-8EF0-BBE88085B03D}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="zbz_no_catalogue_content" localSheetId="0">Tabelle1!$A$1:$D$13</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -35,73 +38,117 @@
 </workbook>
 </file>
 
+<file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
+<connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16">
+  <connection id="1" xr16:uid="{746AA14E-FF49-2241-A966-626DDAF7556F}" name="zbz_no_catalogue_content" type="6" refreshedVersion="8" background="1" saveData="1">
+    <textPr sourceFile="/Users/steffen/git/goobi-workflow/plugin-import-zbz-no-catalogue/docs/zbz_no_catalogue_content.csv" decimal="," thousands=".">
+      <textFields count="3">
+        <textField/>
+        <textField/>
+        <textField/>
+      </textFields>
+    </textPr>
+  </connection>
+</connections>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="32">
+  <si>
+    <t>990056458180205000_1952</t>
+  </si>
+  <si>
+    <t>LGS 50</t>
+  </si>
   <si>
     <t>Title of volume 1952</t>
   </si>
   <si>
-    <t>varia</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Title of volume 1953</t>
-  </si>
-  <si>
-    <t>LGS 50</t>
+    <t>990056458180205000_1953</t>
+  </si>
+  <si>
+    <t>Title of volume 1953</t>
+  </si>
+  <si>
+    <t>990056458180205000_1954</t>
+  </si>
+  <si>
+    <t>Title of volume 1954</t>
+  </si>
+  <si>
+    <t>990056458180205000_1955</t>
+  </si>
+  <si>
+    <t>Title of volume 1955</t>
+  </si>
+  <si>
+    <t>990056458180205000_1956</t>
+  </si>
+  <si>
+    <t>Title of volume 1956</t>
+  </si>
+  <si>
+    <t>990056123423000</t>
+  </si>
+  <si>
+    <t>X1Y2Z3</t>
+  </si>
+  <si>
+    <t>Title of monograph</t>
+  </si>
+  <si>
+    <t>990056458180205000_1957</t>
+  </si>
+  <si>
+    <t>Title of volume 1957</t>
+  </si>
+  <si>
+    <t>990056458180205000_1958</t>
+  </si>
+  <si>
+    <t>Title of volume 1958</t>
+  </si>
+  <si>
+    <t>990056458180205000_1959</t>
+  </si>
+  <si>
+    <t>Title of volume 1959</t>
+  </si>
+  <si>
+    <t>990056458180205000_1960</t>
+  </si>
+  <si>
+    <t>Title of volume 1960</t>
+  </si>
+  <si>
+    <t>990056458180205000_1961</t>
+  </si>
+  <si>
+    <t>Title of volume 1961</t>
+  </si>
+  <si>
+    <t>990056458180205000_1962</t>
+  </si>
+  <si>
+    <t>Title of volume 1962</t>
+  </si>
+  <si>
+    <t>990056458180205000_1963</t>
+  </si>
+  <si>
+    <t>Title of volume 1963</t>
+  </si>
+  <si>
+    <t>Varia</t>
   </si>
   <si>
     <t>dc_bilder</t>
   </si>
   <si>
-    <t>Title of volume 1954</t>
-  </si>
-  <si>
     <t>dc_atlanten</t>
   </si>
   <si>
-    <t>990056458180205000_1954</t>
-  </si>
-  <si>
-    <t>990056458180205000_1953</t>
-  </si>
-  <si>
-    <t>990056458180205000_1952</t>
-  </si>
-  <si>
-    <t>Title of volume 1955</t>
-  </si>
-  <si>
     <t>dc_ch17</t>
-  </si>
-  <si>
-    <t>990056458180205000_1955</t>
-  </si>
-  <si>
-    <t>Title of volume 1956</t>
-  </si>
-  <si>
-    <t>990056458180205000_1956</t>
-  </si>
-  <si>
-    <t>Title of monograph</t>
-  </si>
-  <si>
-    <t>990056123423000</t>
-  </si>
-  <si>
-    <t>X1Y2Z3</t>
-  </si>
-  <si>
-    <t>Title of volume 1957</t>
-  </si>
-  <si>
-    <t>990056458180205000_1957</t>
-  </si>
-  <si>
-    <t>Title of volume 1958</t>
-  </si>
-  <si>
-    <t>990056458180205000_1958</t>
   </si>
 </sst>
 </file>
@@ -112,7 +159,7 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -157,6 +204,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="zbz_no_catalogue_content" connectionId="1" xr16:uid="{468E8DF5-E14A-9F44-B3DA-3D48727F27DE}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
@@ -168,39 +219,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -252,7 +303,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -363,6 +414,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -371,13 +429,6 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -442,158 +493,179 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5404AAA8-2652-9841-98D0-2335DACAA37A}">
-  <dimension ref="A1:D8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB0BAB0F-E333-A541-BFEF-1DD45CC53F85}">
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="66" style="1" customWidth="1"/>
-    <col min="2" max="2" width="25" style="1" customWidth="1"/>
-    <col min="3" max="3" width="23.5" style="1" customWidth="1"/>
-    <col min="4" max="4" width="32.1640625" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="1" width="33.33203125" customWidth="1"/>
+    <col min="2" max="3" width="16.33203125" customWidth="1"/>
+    <col min="4" max="4" width="28.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
         <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" t="s">
         <v>4</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" t="s">
         <v>6</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>15</v>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" t="s">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>20</v>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D13" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>